<commit_message>
Reserved space for SNIPE in drifter log.
</commit_message>
<xml_diff>
--- a/drifter/Drifter_TFO_deployment_log.xlsx
+++ b/drifter/Drifter_TFO_deployment_log.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alaferri/GIT/sio_code/ThodeLab/drifter/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thode/Desktop/ThodeLab/drifter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38A5708E-8625-C644-9142-7C02BEBE3344}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5C08D5D-FCEA-F041-900E-53DD7CF9621B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="840" windowWidth="30240" windowHeight="22120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Drifter Log 2022-2025" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="150">
   <si>
     <t>Deployment</t>
   </si>
@@ -490,18 +490,20 @@
   <si>
     <t>Magnetic Declination</t>
   </si>
+  <si>
+    <t>2025_Oct_CA</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="6">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\Thh:mm:ss"/>
     <numFmt numFmtId="165" formatCode="h:mm;@"/>
     <numFmt numFmtId="166" formatCode="h:mm:ss;@"/>
     <numFmt numFmtId="167" formatCode="0.00000000"/>
     <numFmt numFmtId="168" formatCode="yyyymmdd\Thhmmss"/>
-    <numFmt numFmtId="169" formatCode="hh:mm:ss"/>
   </numFmts>
   <fonts count="16" x14ac:knownFonts="1">
     <font>
@@ -613,7 +615,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -650,6 +652,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -680,7 +688,7 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
@@ -907,9 +915,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="169" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="168" fontId="1" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -920,6 +925,30 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="21" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent3" xfId="1" builtinId="38"/>
@@ -6059,16 +6088,16 @@
       <c r="E49" s="68">
         <v>45780</v>
       </c>
-      <c r="F49" s="86">
+      <c r="F49" s="46">
         <v>0.50486111111111109</v>
       </c>
-      <c r="G49" s="87" t="s">
+      <c r="G49" s="86" t="s">
         <v>141</v>
       </c>
       <c r="H49" s="44">
         <v>20.020324074074075</v>
       </c>
-      <c r="I49" s="88">
+      <c r="I49" s="87">
         <v>-156.00538</v>
       </c>
       <c r="J49" s="45">
@@ -6101,19 +6130,19 @@
       <c r="S49" s="52">
         <v>45780.951365740744</v>
       </c>
-      <c r="T49" s="89">
+      <c r="T49" s="88">
         <v>20.032706000000001</v>
       </c>
-      <c r="U49" s="89">
+      <c r="U49" s="88">
         <v>-155.999832</v>
       </c>
       <c r="V49" s="52">
         <v>45781.875567129631</v>
       </c>
-      <c r="W49" s="89">
+      <c r="W49" s="88">
         <v>20.074359999999999</v>
       </c>
-      <c r="X49" s="89">
+      <c r="X49" s="88">
         <v>-155.953611</v>
       </c>
       <c r="Y49" s="49">
@@ -6147,16 +6176,16 @@
       <c r="E50" s="68">
         <v>45780</v>
       </c>
-      <c r="F50" s="86">
+      <c r="F50" s="46">
         <v>0.50486111111111109</v>
       </c>
-      <c r="G50" s="87" t="s">
+      <c r="G50" s="86" t="s">
         <v>141</v>
       </c>
       <c r="H50" s="44">
         <v>20.020324074074075</v>
       </c>
-      <c r="I50" s="88">
+      <c r="I50" s="87">
         <v>-156.00538</v>
       </c>
       <c r="J50" s="45">
@@ -6189,19 +6218,19 @@
       <c r="S50" s="52">
         <v>45782.028784722221</v>
       </c>
-      <c r="T50" s="89">
+      <c r="T50" s="88">
         <v>20.127566000000002</v>
       </c>
-      <c r="U50" s="89">
+      <c r="U50" s="88">
         <v>-155.93448900000001</v>
       </c>
       <c r="V50" s="52">
         <v>45782.880578703705</v>
       </c>
-      <c r="W50" s="89">
+      <c r="W50" s="88">
         <v>20.216946</v>
       </c>
-      <c r="X50" s="89">
+      <c r="X50" s="88">
         <v>-155.941529</v>
       </c>
       <c r="Y50" s="49">
@@ -6267,19 +6296,19 @@
       <c r="S51" s="74">
         <v>45784.854861111111</v>
       </c>
-      <c r="T51" s="90">
+      <c r="T51" s="89">
         <v>19.972162000000001</v>
       </c>
-      <c r="U51" s="90">
+      <c r="U51" s="89">
         <v>-156.08393000000001</v>
       </c>
       <c r="V51" s="74">
         <v>45785.979861111111</v>
       </c>
-      <c r="W51" s="90">
+      <c r="W51" s="89">
         <v>19.971561000000001</v>
       </c>
-      <c r="X51" s="90">
+      <c r="X51" s="89">
         <v>-156.05051</v>
       </c>
       <c r="Y51" s="76">
@@ -6337,19 +6366,19 @@
       <c r="S52" s="52">
         <v>45788.225694444445</v>
       </c>
-      <c r="T52" s="89">
+      <c r="T52" s="88">
         <v>19.937816000000002</v>
       </c>
-      <c r="U52" s="89">
+      <c r="U52" s="88">
         <v>-155.78363999999999</v>
       </c>
       <c r="V52" s="52">
         <v>45789.118055555555</v>
       </c>
-      <c r="W52" s="89">
+      <c r="W52" s="88">
         <v>20.028275000000001</v>
       </c>
-      <c r="X52" s="89">
+      <c r="X52" s="88">
         <v>-155.99986999999999</v>
       </c>
       <c r="Y52" s="49">
@@ -6366,10 +6395,18 @@
       <c r="AE52" s="44"/>
     </row>
     <row r="53" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="20"/>
-      <c r="B53" s="20"/>
-      <c r="C53" s="20"/>
-      <c r="D53" s="20"/>
+      <c r="A53" s="20">
+        <v>34</v>
+      </c>
+      <c r="B53" s="20" t="s">
+        <v>149</v>
+      </c>
+      <c r="C53" s="20">
+        <v>5</v>
+      </c>
+      <c r="D53" s="20">
+        <v>1</v>
+      </c>
       <c r="E53" s="21"/>
       <c r="F53" s="22"/>
       <c r="G53" s="22"/>
@@ -6399,10 +6436,18 @@
       <c r="AE53" s="20"/>
     </row>
     <row r="54" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="20"/>
-      <c r="B54" s="20"/>
-      <c r="C54" s="20"/>
-      <c r="D54" s="20"/>
+      <c r="A54" s="20">
+        <v>34</v>
+      </c>
+      <c r="B54" s="20" t="s">
+        <v>149</v>
+      </c>
+      <c r="C54" s="20">
+        <v>5</v>
+      </c>
+      <c r="D54" s="20">
+        <v>2</v>
+      </c>
       <c r="E54" s="21"/>
       <c r="F54" s="22"/>
       <c r="G54" s="22"/>
@@ -6432,10 +6477,18 @@
       <c r="AE54" s="20"/>
     </row>
     <row r="55" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="20"/>
-      <c r="B55" s="20"/>
-      <c r="C55" s="20"/>
-      <c r="D55" s="20"/>
+      <c r="A55" s="20">
+        <v>34</v>
+      </c>
+      <c r="B55" s="20" t="s">
+        <v>149</v>
+      </c>
+      <c r="C55" s="20">
+        <v>5</v>
+      </c>
+      <c r="D55" s="20">
+        <v>3</v>
+      </c>
       <c r="E55" s="21"/>
       <c r="F55" s="22"/>
       <c r="G55" s="22"/>
@@ -6464,104 +6517,128 @@
       <c r="AD55" s="20"/>
       <c r="AE55" s="20"/>
     </row>
-    <row r="56" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="20"/>
-      <c r="B56" s="20"/>
-      <c r="C56" s="20"/>
-      <c r="D56" s="20"/>
-      <c r="E56" s="21"/>
-      <c r="F56" s="22"/>
-      <c r="G56" s="22"/>
-      <c r="H56" s="20"/>
-      <c r="I56" s="20"/>
-      <c r="J56" s="21"/>
-      <c r="K56" s="22"/>
-      <c r="L56" s="22"/>
-      <c r="M56" s="20"/>
-      <c r="N56" s="20"/>
-      <c r="O56" s="20"/>
-      <c r="P56" s="20"/>
-      <c r="Q56" s="23"/>
-      <c r="R56" s="23"/>
-      <c r="S56" s="24"/>
-      <c r="T56" s="20"/>
-      <c r="U56" s="20"/>
-      <c r="V56" s="24"/>
-      <c r="W56" s="20"/>
-      <c r="X56" s="20"/>
-      <c r="Y56" s="25"/>
-      <c r="Z56" s="25"/>
-      <c r="AA56" s="26"/>
-      <c r="AB56" s="26"/>
-      <c r="AC56" s="20"/>
-      <c r="AD56" s="20"/>
-      <c r="AE56" s="20"/>
-    </row>
-    <row r="57" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="20"/>
-      <c r="B57" s="20"/>
-      <c r="C57" s="20"/>
-      <c r="D57" s="20"/>
-      <c r="E57" s="21"/>
-      <c r="F57" s="22"/>
-      <c r="G57" s="22"/>
-      <c r="H57" s="20"/>
-      <c r="I57" s="20"/>
-      <c r="J57" s="21"/>
-      <c r="K57" s="22"/>
-      <c r="L57" s="22"/>
-      <c r="M57" s="20"/>
-      <c r="N57" s="20"/>
-      <c r="O57" s="20"/>
-      <c r="P57" s="20"/>
-      <c r="Q57" s="23"/>
-      <c r="R57" s="23"/>
-      <c r="S57" s="24"/>
-      <c r="T57" s="20"/>
-      <c r="U57" s="20"/>
-      <c r="V57" s="24"/>
-      <c r="W57" s="20"/>
-      <c r="X57" s="20"/>
-      <c r="Y57" s="25"/>
-      <c r="Z57" s="25"/>
-      <c r="AA57" s="26"/>
-      <c r="AB57" s="26"/>
-      <c r="AC57" s="20"/>
-      <c r="AD57" s="20"/>
-      <c r="AE57" s="20"/>
-    </row>
-    <row r="58" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="20"/>
-      <c r="B58" s="20"/>
-      <c r="C58" s="20"/>
-      <c r="D58" s="20"/>
-      <c r="E58" s="21"/>
-      <c r="F58" s="22"/>
-      <c r="G58" s="22"/>
-      <c r="H58" s="20"/>
-      <c r="I58" s="20"/>
-      <c r="J58" s="21"/>
-      <c r="K58" s="22"/>
-      <c r="L58" s="22"/>
-      <c r="M58" s="20"/>
-      <c r="N58" s="20"/>
-      <c r="O58" s="20"/>
-      <c r="P58" s="20"/>
-      <c r="Q58" s="23"/>
-      <c r="R58" s="23"/>
-      <c r="S58" s="24"/>
-      <c r="T58" s="20"/>
-      <c r="U58" s="20"/>
-      <c r="V58" s="24"/>
-      <c r="W58" s="20"/>
-      <c r="X58" s="20"/>
-      <c r="Y58" s="25"/>
-      <c r="Z58" s="25"/>
-      <c r="AA58" s="26"/>
-      <c r="AB58" s="26"/>
-      <c r="AC58" s="20"/>
-      <c r="AD58" s="20"/>
-      <c r="AE58" s="20"/>
+    <row r="56" spans="1:31" s="99" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="92">
+        <v>35</v>
+      </c>
+      <c r="B56" s="92" t="s">
+        <v>149</v>
+      </c>
+      <c r="C56" s="92">
+        <v>6</v>
+      </c>
+      <c r="D56" s="92">
+        <v>1</v>
+      </c>
+      <c r="E56" s="93"/>
+      <c r="F56" s="94"/>
+      <c r="G56" s="94"/>
+      <c r="H56" s="92"/>
+      <c r="I56" s="92"/>
+      <c r="J56" s="93"/>
+      <c r="K56" s="94"/>
+      <c r="L56" s="94"/>
+      <c r="M56" s="92"/>
+      <c r="N56" s="92"/>
+      <c r="O56" s="92"/>
+      <c r="P56" s="92"/>
+      <c r="Q56" s="95"/>
+      <c r="R56" s="95"/>
+      <c r="S56" s="96"/>
+      <c r="T56" s="92"/>
+      <c r="U56" s="92"/>
+      <c r="V56" s="96"/>
+      <c r="W56" s="92"/>
+      <c r="X56" s="92"/>
+      <c r="Y56" s="97"/>
+      <c r="Z56" s="97"/>
+      <c r="AA56" s="98"/>
+      <c r="AB56" s="98"/>
+      <c r="AC56" s="92"/>
+      <c r="AD56" s="92"/>
+      <c r="AE56" s="92"/>
+    </row>
+    <row r="57" spans="1:31" s="99" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="92">
+        <v>35</v>
+      </c>
+      <c r="B57" s="92" t="s">
+        <v>149</v>
+      </c>
+      <c r="C57" s="92">
+        <v>6</v>
+      </c>
+      <c r="D57" s="92">
+        <v>2</v>
+      </c>
+      <c r="E57" s="93"/>
+      <c r="F57" s="94"/>
+      <c r="G57" s="94"/>
+      <c r="H57" s="92"/>
+      <c r="I57" s="92"/>
+      <c r="J57" s="93"/>
+      <c r="K57" s="94"/>
+      <c r="L57" s="94"/>
+      <c r="M57" s="92"/>
+      <c r="N57" s="92"/>
+      <c r="O57" s="92"/>
+      <c r="P57" s="92"/>
+      <c r="Q57" s="95"/>
+      <c r="R57" s="95"/>
+      <c r="S57" s="96"/>
+      <c r="T57" s="92"/>
+      <c r="U57" s="92"/>
+      <c r="V57" s="96"/>
+      <c r="W57" s="92"/>
+      <c r="X57" s="92"/>
+      <c r="Y57" s="97"/>
+      <c r="Z57" s="97"/>
+      <c r="AA57" s="98"/>
+      <c r="AB57" s="98"/>
+      <c r="AC57" s="92"/>
+      <c r="AD57" s="92"/>
+      <c r="AE57" s="92"/>
+    </row>
+    <row r="58" spans="1:31" s="99" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="92">
+        <v>35</v>
+      </c>
+      <c r="B58" s="92" t="s">
+        <v>149</v>
+      </c>
+      <c r="C58" s="92">
+        <v>6</v>
+      </c>
+      <c r="D58" s="92">
+        <v>3</v>
+      </c>
+      <c r="E58" s="93"/>
+      <c r="F58" s="94"/>
+      <c r="G58" s="94"/>
+      <c r="H58" s="92"/>
+      <c r="I58" s="92"/>
+      <c r="J58" s="93"/>
+      <c r="K58" s="94"/>
+      <c r="L58" s="94"/>
+      <c r="M58" s="92"/>
+      <c r="N58" s="92"/>
+      <c r="O58" s="92"/>
+      <c r="P58" s="92"/>
+      <c r="Q58" s="95"/>
+      <c r="R58" s="95"/>
+      <c r="S58" s="96"/>
+      <c r="T58" s="92"/>
+      <c r="U58" s="92"/>
+      <c r="V58" s="96"/>
+      <c r="W58" s="92"/>
+      <c r="X58" s="92"/>
+      <c r="Y58" s="97"/>
+      <c r="Z58" s="97"/>
+      <c r="AA58" s="98"/>
+      <c r="AB58" s="98"/>
+      <c r="AC58" s="92"/>
+      <c r="AD58" s="92"/>
+      <c r="AE58" s="92"/>
     </row>
     <row r="59" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="20"/>
@@ -48056,11 +48133,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" ht="96" x14ac:dyDescent="0.2">
-      <c r="A1" s="91" t="s">
+      <c r="A1" s="90" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="92"/>
-      <c r="C1" s="92"/>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
       <c r="D1" s="9" t="s">
         <v>53</v>
       </c>

</xml_diff>